<commit_message>
Remove API question from migration questions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F9SjPdqWc4obrbWGcH8Ho7
</commit_message>
<xml_diff>
--- a/Fabulate_4_Platform_Migration_Questions.xlsx
+++ b/Fabulate_4_Platform_Migration_Questions.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -510,7 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What campaign data can move from the old platform to the new one, and how can APIs and AI reduce CM workload? Dev team to fill in the yellow columns.</t>
+          <t>What campaign data can move from the old platform to the new one, and how can we reduce CM workload? Dev team to fill in the yellow columns.</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Does the old platform have an API or database export we can pull campaign data from, and can the new platform take it in via API?</t>
+          <t>Which parts of the migration can be fully automated, which can be AI-assisted with CM review, and which will stay manual?</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -570,12 +570,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Approach</t>
+          <t>Campaigns</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Which parts of the migration can be fully automated, which can be AI-assisted with CM review, and which will stay manual?</t>
+          <t>Which campaign details can move across automatically (name, client, CM lead, team, dates, budget, deliverables)?</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -593,7 +593,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Which campaign details can move across automatically (name, client, CM lead, team, dates, budget, deliverables)?</t>
+          <t>Can we migrate live campaigns first and keep completed ones as a read-only archive?</t>
         </is>
       </c>
       <c r="D7" s="5" t="n"/>
@@ -606,12 +606,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Campaigns</t>
+          <t>Briefs</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Can we migrate live campaigns first and keep completed ones as a read-only archive?</t>
+          <t>Can briefs move across with full content and attachments intact, still linked to their campaign?</t>
         </is>
       </c>
       <c r="D8" s="5" t="n"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Can briefs move across with full content and attachments intact, still linked to their campaign?</t>
+          <t>If the new brief format is different, can AI map the old brief text into the new brief fields for CMs to review?</t>
         </is>
       </c>
       <c r="D9" s="5" t="n"/>
@@ -642,12 +642,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Briefs</t>
+          <t>Creators</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>If the new brief format is different, can AI map the old brief text into the new brief fields for CMs to review?</t>
+          <t>Can creator profiles move across, and how will duplicate creators be handled?</t>
         </is>
       </c>
       <c r="D10" s="5" t="n"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Can creator profiles move across, and how will duplicate creators be handled?</t>
+          <t>Will each creator stay linked to the right brief and campaign, with their agreed fee, deliverables and usage rights?</t>
         </is>
       </c>
       <c r="D11" s="5" t="n"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Will each creator stay linked to the right brief and campaign, with their agreed fee, deliverables and usage rights?</t>
+          <t>Will creators need to re-register or re-accept terms on the new platform?</t>
         </is>
       </c>
       <c r="D12" s="5" t="n"/>
@@ -696,12 +696,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Creators</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Will creators need to re-register or re-accept terms on the new platform?</t>
+          <t>Can each creator's current stage on a campaign be migrated, and do the old and new status stages match?</t>
         </is>
       </c>
       <c r="D13" s="5" t="n"/>
@@ -719,7 +719,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Can each creator's current stage on a campaign be migrated, and do the old and new status stages match?</t>
+          <t>How will in-flight work be handled (drafts in review, pending approvals, unpaid creators)?</t>
         </is>
       </c>
       <c r="D14" s="5" t="n"/>
@@ -732,12 +732,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Comments</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>How will in-flight work be handled (drafts in review, pending approvals, unpaid creators)?</t>
+          <t>Can comment threads move across with author, date and attachments, still attached to the right creator, brief or content?</t>
         </is>
       </c>
       <c r="D15" s="5" t="n"/>
@@ -755,7 +755,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Can comment threads move across with author, date and attachments, still attached to the right creator, brief or content?</t>
+          <t>If full comments cannot move, can AI summarise each thread (key feedback, approvals, open actions)?</t>
         </is>
       </c>
       <c r="D16" s="5" t="n"/>
@@ -768,12 +768,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Comments</t>
+          <t>Vault</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>If full comments cannot move, can AI summarise each thread (key feedback, approvals, open actions)?</t>
+          <t>Can Vault files (videos, concepts, drafts, finals) be bulk transferred, rather than CMs downloading and re-uploading?</t>
         </is>
       </c>
       <c r="D17" s="5" t="n"/>
@@ -791,7 +791,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Can Vault files (videos, concepts, drafts, finals) be bulk transferred, rather than CMs downloading and re-uploading?</t>
+          <t>Will file details come with them (creator, campaign, version, approval status, usage rights)?</t>
         </is>
       </c>
       <c r="D18" s="5" t="n"/>
@@ -804,12 +804,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Vault</t>
+          <t>Data safety</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Will file details come with them (creator, campaign, version, approval status, usage rights)?</t>
+          <t>How will client and creator data be kept secure and confidential during migration, including any AI tools used?</t>
         </is>
       </c>
       <c r="D19" s="5" t="n"/>
@@ -822,12 +822,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Data safety</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>How will client and creator data be kept secure and confidential during migration, including any AI tools used?</t>
+          <t>Can we pilot the migration on one or two campaigns first so CMs can check the result?</t>
         </is>
       </c>
       <c r="D20" s="5" t="n"/>
@@ -845,7 +845,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Can we pilot the migration on one or two campaigns first so CMs can check the result?</t>
+          <t>Will there be a report showing what moved, what failed and what CMs need to fix manually?</t>
         </is>
       </c>
       <c r="D21" s="5" t="n"/>
@@ -858,12 +858,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Cutover</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Will there be a report showing what moved, what failed and what CMs need to fix manually?</t>
+          <t>Will there be a freeze period on the old platform, and how will changes made during migration be captured?</t>
         </is>
       </c>
       <c r="D22" s="5" t="n"/>
@@ -881,33 +881,15 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Will there be a freeze period on the old platform, and how will changes made during migration be captured?</t>
+          <t>What is the timeline, how long will the old platform stay accessible, and what do CMs need to do at each stage?</t>
         </is>
       </c>
       <c r="D23" s="5" t="n"/>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Cutover</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>What is the timeline, how long will the old platform stay accessible, and what do CMs need to do at each stage?</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="D5:D24">
+  <conditionalFormatting sqref="D5:D23">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>D5="Yes"</formula>
     </cfRule>
@@ -919,11 +901,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="D5:D24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,Partial,No,TBC"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"API,AI assisted,API + AI,Manual,TBC"</formula1>
+    <dataValidation sqref="E5:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Automated,AI assisted,Manual,TBC"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refocus migration questions on tasks, briefs, creators, contracts and client comms
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F9SjPdqWc4obrbWGcH8Ho7
</commit_message>
<xml_diff>
--- a/Fabulate_4_Platform_Migration_Questions.xlsx
+++ b/Fabulate_4_Platform_Migration_Questions.xlsx
@@ -493,7 +493,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="75" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -552,12 +552,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Approach</t>
+          <t>Campaign tasks</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Which parts of the migration can be fully automated, which can be AI-assisted with CM review, and which will stay manual?</t>
+          <t>Can campaign tasks be migrated with their details (task name, assignee, due date, status)?</t>
         </is>
       </c>
       <c r="D5" s="5" t="n"/>
@@ -570,12 +570,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Campaigns</t>
+          <t>Campaign tasks</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Which campaign details can move across automatically (name, client, CM lead, team, dates, budget, deliverables)?</t>
+          <t>Will tasks stay linked to the correct campaign, brief and creator?</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -588,12 +588,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Campaigns</t>
+          <t>Campaign tasks</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Can we migrate live campaigns first and keep completed ones as a read-only archive?</t>
+          <t>Can completed tasks come across as history, or only open tasks?</t>
         </is>
       </c>
       <c r="D7" s="5" t="n"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Can briefs move across with full content and attachments intact, still linked to their campaign?</t>
+          <t>Can briefs be migrated with their full content and attachments intact?</t>
         </is>
       </c>
       <c r="D8" s="5" t="n"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>If the new brief format is different, can AI map the old brief text into the new brief fields for CMs to review?</t>
+          <t>Will each brief stay linked to its campaign?</t>
         </is>
       </c>
       <c r="D9" s="5" t="n"/>
@@ -642,12 +642,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Creators</t>
+          <t>Briefs</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Can creator profiles move across, and how will duplicate creators be handled?</t>
+          <t>If the new brief format is different, can AI map the old brief text into the new brief fields for CMs to review?</t>
         </is>
       </c>
       <c r="D10" s="5" t="n"/>
@@ -660,12 +660,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Creators</t>
+          <t>Influencers on briefs</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Will each creator stay linked to the right brief and campaign, with their agreed fee, deliverables and usage rights?</t>
+          <t>Can the influencers attached to each brief be migrated, keeping the link to that brief?</t>
         </is>
       </c>
       <c r="D11" s="5" t="n"/>
@@ -678,12 +678,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Creators</t>
+          <t>Influencers on briefs</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Will creators need to re-register or re-accept terms on the new platform?</t>
+          <t>Will each influencer's current status on the brief come across (e.g. invited, accepted, draft submitted, approved, live)?</t>
         </is>
       </c>
       <c r="D12" s="5" t="n"/>
@@ -696,12 +696,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Influencers on briefs</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Can each creator's current stage on a campaign be migrated, and do the old and new status stages match?</t>
+          <t>How will influencers who sit on multiple briefs be handled so they are not duplicated?</t>
         </is>
       </c>
       <c r="D13" s="5" t="n"/>
@@ -714,12 +714,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Budget / contract</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>How will in-flight work be handled (drafts in review, pending approvals, unpaid creators)?</t>
+          <t>Can the agreed fee or budget for each creator be migrated?</t>
         </is>
       </c>
       <c r="D14" s="5" t="n"/>
@@ -732,12 +732,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Comments</t>
+          <t>Budget / contract</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Can comment threads move across with author, date and attachments, still attached to the right creator, brief or content?</t>
+          <t>Can the contract attached to each creator come across (deliverables, usage rights, exclusivity, T&amp;C acceptance)?</t>
         </is>
       </c>
       <c r="D15" s="5" t="n"/>
@@ -750,12 +750,12 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Comments</t>
+          <t>Budget / contract</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>If full comments cannot move, can AI summarise each thread (key feedback, approvals, open actions)?</t>
+          <t>Will payment status for each creator (invoiced, paid, unpaid) be migrated?</t>
         </is>
       </c>
       <c r="D16" s="5" t="n"/>
@@ -768,12 +768,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Vault</t>
+          <t>Internal tasks</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Can Vault files (videos, concepts, drafts, finals) be bulk transferred, rather than CMs downloading and re-uploading?</t>
+          <t>Can internal tasks be migrated with their assignee, due date and status?</t>
         </is>
       </c>
       <c r="D17" s="5" t="n"/>
@@ -786,12 +786,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Vault</t>
+          <t>Internal tasks</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Will file details come with them (creator, campaign, version, approval status, usage rights)?</t>
+          <t>Will internal tasks stay internal, so clients and creators cannot see them on the new platform?</t>
         </is>
       </c>
       <c r="D18" s="5" t="n"/>
@@ -804,12 +804,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Data safety</t>
+          <t>Internal tasks</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>How will client and creator data be kept secure and confidential during migration, including any AI tools used?</t>
+          <t>Can internal notes or comments on tasks come across?</t>
         </is>
       </c>
       <c r="D19" s="5" t="n"/>
@@ -822,12 +822,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Client comms (Odin)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Can we pilot the migration on one or two campaigns first so CMs can check the result?</t>
+          <t>How are clients currently engaging with us on Odin (comments, approvals, messages, notifications, reports)?</t>
         </is>
       </c>
       <c r="D20" s="5" t="n"/>
@@ -840,12 +840,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Client comms (Odin)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Will there be a report showing what moved, what failed and what CMs need to fix manually?</t>
+          <t>Can client comments and approval history on content be migrated?</t>
         </is>
       </c>
       <c r="D21" s="5" t="n"/>
@@ -858,12 +858,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Cutover</t>
+          <t>Client comms (Odin)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Will there be a freeze period on the old platform, and how will changes made during migration be captured?</t>
+          <t>Can client message threads be migrated, still linked to the right campaign, brief or content?</t>
         </is>
       </c>
       <c r="D22" s="5" t="n"/>
@@ -876,12 +876,12 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Cutover</t>
+          <t>Client comms (Odin)</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>What is the timeline, how long will the old platform stay accessible, and what do CMs need to do at each stage?</t>
+          <t>If full client comms history cannot come across, can AI summarise it for each campaign?</t>
         </is>
       </c>
       <c r="D23" s="5" t="n"/>

</xml_diff>